<commit_message>
perf: optimize supplier lookup by pre-computing data to eliminate O(N^3) complexity in export loop
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -4,17 +4,22 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="test" state="visible" r:id="rId3"/>
+    <sheet sheetId="1" name="Test" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+  <si>
+    <t>A</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -44,9 +49,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -389,12 +393,12 @@
   <dimension ref="A1:A1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="9" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1">
-        <v>45900.875</v>
+      <c r="A1" t="s">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -666,13 +670,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CC8DAEE2-1E7F-45D2-9692-7438D9739DDC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F86CE3B4-8742-4132-8E84-86C6A8B22D59}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8A5425F-956F-4702-87C6-1E1253460250}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC75E664-6EB2-4683-87BE-07A79FECF1D0}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F89C791C-6AA7-427C-8A00-7886EB54F0B0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83F22EA3-5AE4-4961-88AD-08D1277F34D5}"/>
 </file>
</xml_diff>

<commit_message>
chore: update test spreadsheet and generate debug log file
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -13,13 +13,16 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
-    <t>A</t>
+    <t>Date</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yy"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
@@ -49,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -390,15 +394,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="6.5" customWidth="1"/>
+    <col min="1" max="1" width="7.6" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>45901.5</v>
       </c>
     </row>
   </sheetData>
@@ -670,13 +679,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F86CE3B4-8742-4132-8E84-86C6A8B22D59}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C5FC454D-91FC-4230-B144-1C9FA7F5BC3C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BC75E664-6EB2-4683-87BE-07A79FECF1D0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58BB5E78-4395-4158-AF4C-E5EA62E1BEFF}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83F22EA3-5AE4-4961-88AD-08D1277F34D5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AFAB4FC3-B7C9-4499-8C1D-DC3BFEA5818F}"/>
 </file>
</xml_diff>